<commit_message>
Add carousel-hero block, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (6):
- blocks/carousel-hero/carousel-hero.css
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/index.report.json
- tools/importer/transformers/albertsons-cleanup.js
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>index.report.json</t>
   </si>
   <si>
-    <t>["cards-category","cards-banner","cards-banner","cards-banner","cards-banner","cards-banner","cards-banner","cards-banner","cards-banner","cards-banner"]</t>
+    <t>["cards-banner","cards-banner","cards-banner","cards-banner","cards-banner","cards-banner","cards-banner","cards-banner","cards-banner"]</t>
   </si>
   <si>
     <t>index</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-04-08T04:10:47.224Z</t>
+    <t>2026-04-08T04:45:52.666Z</t>
   </si>
   <si>
     <t>Grocery Delivery Near You - Order Groceries Online | Albertsons</t>

</xml_diff>